<commit_message>
finance-portfolio: fix overlapping charts, add real number formatting to XLS report
Charts sheet anchored the pie and line charts too close together (pie's
rendered height exceeded the row gap before the trend table started),
causing visual overlap. Charts are now anchored with a fixed clearance
computed from the pie's actual rendered size, and both charts are
bigger and carry proper titles/legends/data labels.

Also replaced flat, unformatted numbers across every sheet with real
currency/percent number formats, banded rows, colored G/L and sleeve-
drift deltas, a KPI-card cover layout, and a sleeve target-vs-current
bar chart on the Summary tab — the report no longer looks like a bare
data dump.
</commit_message>
<xml_diff>
--- a/quarterly-reports/2026-starting-book.xlsx
+++ b/quarterly-reports/2026-starting-book.xlsx
@@ -20,8 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="8">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_($* #,##0.00_);_($* (#,##0.00);_($* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="+0.00%;-0.00%"/>
+  </numFmts>
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,43 +33,87 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5496"/>
-      <sz val="18"/>
+      <color rgb="001F3864"/>
+      <sz val="20"/>
     </font>
     <font>
       <i val="1"/>
-      <sz val="11"/>
+      <color rgb="002F5496"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F3864"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00777777"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5496"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002F5496"/>
-      <sz val="14"/>
+      <color rgb="00C62828"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E7D32"/>
+    </font>
+    <font>
+      <color rgb="002E7D32"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002F5496"/>
-      <sz val="12"/>
+      <color rgb="00E67E22"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -76,12 +123,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6DCE4"/>
-        <bgColor rgb="00D6DCE4"/>
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F6FB"/>
+        <bgColor rgb="00F2F6FB"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -90,34 +143,140 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00B9C6D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B9C6D6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B9C6D6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B9C6D6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F3864"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="14" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="00C62828"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -192,6 +351,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -202,7 +362,130 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Theme Exposure</a:t>
+              <a:t>Sleeve Allocation: Target vs. Current</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!B10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$A$11:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$11:$B$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Summary'!C10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$A$11:$A$15</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$C$11:$C$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% of NAV</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="26"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Theme Exposure (% NAV)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -216,7 +499,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Charts'!B1</f>
+              <f>'Charts'!B3</f>
             </strRef>
           </tx>
           <spPr>
@@ -226,15 +509,18 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Charts'!$A$2:$A$8</f>
+              <f>'Charts'!$A$4:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$2:$B$8</f>
+              <f>'Charts'!$B$4:$B$10</f>
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>
@@ -247,8 +533,9 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
   <chart>
     <title>
       <tx>
@@ -273,7 +560,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Charts'!B11</f>
+              <f>'Charts'!B26</f>
             </strRef>
           </tx>
           <spPr>
@@ -282,7 +569,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="5"/>
             <spPr>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -291,21 +579,22 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$12:$A$13</f>
+              <f>'Charts'!$A$27:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$B$12:$B$13</f>
+              <f>'Charts'!$B$27:$B$28</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="1"/>
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Charts'!C11</f>
+              <f>'Charts'!C26</f>
             </strRef>
           </tx>
           <spPr>
@@ -314,7 +603,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="5"/>
             <spPr>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -323,21 +613,22 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$12:$A$13</f>
+              <f>'Charts'!$A$27:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$C$12:$C$13</f>
+              <f>'Charts'!$C$27:$C$28</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <ser>
           <idx val="2"/>
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Charts'!D11</f>
+              <f>'Charts'!D26</f>
             </strRef>
           </tx>
           <spPr>
@@ -346,7 +637,8 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="5"/>
             <spPr>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -355,14 +647,15 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Charts'!$A$12:$A$13</f>
+              <f>'Charts'!$A$27:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Charts'!$D$12:$D$13</f>
+              <f>'Charts'!$D$27:$D$28</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -373,6 +666,21 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Cycle Date</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -385,13 +693,28 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Value</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -403,12 +726,39 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>0</row>
+      <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5760000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -427,10 +777,10 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="7920000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -737,86 +1087,99 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A2:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>PORTFOLIO PERFORMANCE REPORT</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Period: Starting Book — as of 2026-09-05 (Cycle #2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="E2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Starting Book — as of 2026-09-05 (Cycle #2)</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Prepared for: Mr. Spock — Logical Investor</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>A hypothetical growth-oriented investor in the accumulation phase, governed by a fixed sizing table, a 25% theme-concentration cap, and a wall-clock-derived glide path. See investor-profile.md for the full mandate. Zero real personal data underlies this profile.</t>
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7"/>
     <row r="8"/>
     <row r="9"/>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Glide-Path Phase</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Cycle #</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="B12" s="7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Accumulation</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Cycle #</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+      <c r="D12" s="8" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>IMPORTANT: This is a paper/model portfolio for evaluation purposes only, tracked with public market data alone (no personal financial context). It does not constitute investment advice or a recommendation to buy or sell any security. All investments involve risk, including potential loss of principal. Always consult with qualified financial professionals before making investment decisions.</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A5:D8"/>
-    <mergeCell ref="A13:D16"/>
+  <mergeCells count="5">
+    <mergeCell ref="B6:D9"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B15:D19"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -828,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -837,8 +1200,8 @@
     <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>SUMMARY</t>
         </is>
@@ -846,175 +1209,190 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>This Portfolio</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Blended Benchmark</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>NAV</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="13" t="n">
         <v>100000</v>
       </c>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Period Return %</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="n">
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Since-Inception Return %</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D6" t="n">
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7"/>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>SLEEVE DRIFT VS. TARGET</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Sleeve</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Target %</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Current %</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Drift</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Individual Stocks</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C11" s="16" t="n">
         <v>0.4906</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" s="18" t="n">
         <v>-0.009400000000000019</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Sector ETFs</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" s="15" t="n">
         <v>0.2</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.1655</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" s="20" t="n">
         <v>-0.0345</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Hedge (GLD/IAU)</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B13" s="16" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" s="18" t="n">
         <v>-0.07000000000000001</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Bonds (AGG)</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B14" s="15" t="n">
         <v>0.13</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C14" s="15" t="n">
         <v>0.0803</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" s="20" t="n">
         <v>-0.04970000000000001</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Cash (floor 10%)</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B15" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C15" s="16" t="n">
         <v>0.2637</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" s="21" t="n">
         <v>0.1637</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D11:D15">
+    <cfRule type="dataBar" priority="1">
+      <dataBar showValue="1">
+        <cfvo type="num" val="-0.15"/>
+        <cfvo type="num" val="0.15"/>
+        <color rgb="00F4B183"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1024,7 +1402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1038,532 +1416,568 @@
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>HOLDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Mkt Value</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>% NAV</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>Unrealized G/L</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D4" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E4" s="13" t="n">
         <v>357.56</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F4" s="13" t="n">
         <v>357.56</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G4" s="13" t="n">
         <v>5005.84</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H4" s="16" t="n">
         <v>0.0501</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I4" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>ETN</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Energy-Transition</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D5" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E5" s="27" t="n">
         <v>412.97</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F5" s="27" t="n">
         <v>412.97</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G5" s="27" t="n">
         <v>4955.64</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H5" s="15" t="n">
         <v>0.0496</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I5" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>COF</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D6" s="23" t="n">
         <v>23</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E6" s="13" t="n">
         <v>216.96</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F6" s="13" t="n">
         <v>216.96</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G6" s="13" t="n">
         <v>4990.08</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H6" s="16" t="n">
         <v>0.0499</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I6" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>LLY</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Healthcare-GLP1</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D7" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E7" s="27" t="n">
         <v>1215.13</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F7" s="27" t="n">
         <v>1215.13</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G7" s="27" t="n">
         <v>4860.52</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H7" s="15" t="n">
         <v>0.0486</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I7" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>TJX</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Consumer-Defensive</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D8" s="23" t="n">
         <v>35</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E8" s="13" t="n">
         <v>139.48</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F8" s="13" t="n">
         <v>139.48</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G8" s="13" t="n">
         <v>4881.8</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H8" s="16" t="n">
         <v>0.0488</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I8" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>GOOGL</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D9" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E9" s="27" t="n">
         <v>341.95</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F9" s="27" t="n">
         <v>341.95</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G9" s="27" t="n">
         <v>4787.3</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H9" s="15" t="n">
         <v>0.0479</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I9" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>BALL</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D10" s="23" t="n">
         <v>81</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E10" s="13" t="n">
         <v>61.3</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F10" s="13" t="n">
         <v>61.3</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G10" s="13" t="n">
         <v>4965.3</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H10" s="16" t="n">
         <v>0.0497</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I10" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Consumer-Defensive</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D11" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E11" s="27" t="n">
         <v>142.27</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F11" s="27" t="n">
         <v>142.27</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G11" s="27" t="n">
         <v>4979.45</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H11" s="15" t="n">
         <v>0.0498</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I11" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>NEE</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D12" s="23" t="n">
         <v>59</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E12" s="13" t="n">
         <v>84.29000000000001</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F12" s="13" t="n">
         <v>84.29000000000001</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G12" s="13" t="n">
         <v>4973.11</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H12" s="16" t="n">
         <v>0.0497</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I12" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D13" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E13" s="27" t="n">
         <v>930.25</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F13" s="27" t="n">
         <v>930.25</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G13" s="27" t="n">
         <v>4651.25</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H13" s="15" t="n">
         <v>0.0465</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I13" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>XLK</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Sector ETF</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E14" s="13" t="n">
         <v>186</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F14" s="13" t="n">
         <v>186</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G14" s="13" t="n">
         <v>5580</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H14" s="16" t="n">
         <v>0.0558</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I14" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>XLI</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Sector ETF</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Energy-Transition</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D15" s="26" t="n">
         <v>59</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E15" s="27" t="n">
         <v>185.96</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F15" s="27" t="n">
         <v>185.96</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G15" s="27" t="n">
         <v>10971.64</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H15" s="15" t="n">
         <v>0.1097</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I15" s="28" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>AGG</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Bond</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Diversified-Core</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D16" s="23" t="n">
         <v>82</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E16" s="13" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F16" s="13" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G16" s="13" t="n">
         <v>8027.8</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H16" s="16" t="n">
         <v>0.0803</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I16" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G15" t="n">
+      <c r="D17" s="26" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n">
         <v>26370.27</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H17" s="15" t="n">
         <v>0.2637</v>
       </c>
+      <c r="I17" s="27" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n"/>
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n"/>
+      <c r="F18" s="29" t="n"/>
+      <c r="G18" s="30" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H18" s="31" t="n">
+        <v>1.0001</v>
+      </c>
+      <c r="I18" s="29" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="I4:I17">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1574,7 +1988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1585,425 +1999,433 @@
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>TRADE LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>XLK</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" s="32" t="inlineStr">
         <is>
           <t>TRIM</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D4" s="23" t="n">
         <v>-29</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E4" s="13" t="n">
         <v>186</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>Rebalance — rules change (not a thesis exit). Introduced the 25% theme-concentration cap; AI-Capex (AVGO, GOOGL, NEE, MU, XLK) had drifted to 30.39% NAV. Trimmed XLK from 59 sh to 30 sh, proceeds routed to cash, bringing AI-Capex to 25.00% NAV. No fundamental thesis changed for any of the five AI-Capex positions.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>LLY</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D5" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E5" s="27" t="n">
         <v>1215.13</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F5" s="35" t="inlineStr">
         <is>
           <t>Q2 2026 revenue +47.7% YoY, EPS beat, raised FY2026 guidance. GLP-1 franchise demand catalyst. Entered on a down day. Stop: guidance cut or GLP-1 share loss.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>TJX</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D6" s="23" t="n">
         <v>35</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E6" s="13" t="n">
         <v>139.48</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F6" s="33" t="inlineStr">
         <is>
           <t>Off-price model delivering 5% comps; steady grower, not chasing an all-time high. Diversification into defensive-leaning consumer discretionary.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>GOOGL</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D7" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E7" s="27" t="n">
         <v>341.95</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F7" s="35" t="inlineStr">
         <is>
           <t>Accelerating Google Cloud AI adoption; BNP Paribas Outperform, $420 target. Entered on a down day. Diversification into communication services.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>BALL</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C8" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D8" s="23" t="n">
         <v>81</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E8" s="13" t="n">
         <v>61.3</v>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>Analysts raised fair-value estimate to $63.26; aluminum-packaging demand recovery. Diversification into materials.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D9" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E9" s="27" t="n">
         <v>142.27</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F9" s="35" t="inlineStr">
         <is>
           <t>Organic volume growth accelerating to +1% as streamlining pays off; trading below 12-month average target. Diversification into consumer staples.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>NEE</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D10" s="23" t="n">
         <v>59</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E10" s="13" t="n">
         <v>84.29000000000001</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F10" s="33" t="inlineStr">
         <is>
           <t>$100B data-center campus JV with Brookfield; 21GW large-load pipeline. Diversification into utilities, direct AI power-demand exposure.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D11" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E11" s="27" t="n">
         <v>930.25</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F11" s="35" t="inlineStr">
         <is>
           <t>Fiscal Q2 revenue +196% YoY; HBM supply sold out for 2026. Morgan Stanley top 2026 semiconductor pick. Second AI-infrastructure name (memory vs. networking).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>XLK</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D12" s="23" t="n">
         <v>59</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E12" s="13" t="n">
         <v>186</v>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F12" s="33" t="inlineStr">
         <is>
           <t>W4 sector-rotation scan: Tech receiving dominant share of 2026 sector inflows, driven by AI capex. Top accumulation-signal sector.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>XLI</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D13" s="26" t="n">
         <v>59</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E13" s="27" t="n">
         <v>185.96</v>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="35" t="inlineStr">
         <is>
           <t>Best-performing S&amp;P sector YTD 2026 (+19.5%); AI-data-center power/cooling capex and reshoring/logistics demand.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E14" s="13" t="n">
         <v>357.56</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Record $22.1B quarterly revenue, 25.2% YoY growth, 54.7% EBITDA margin. AI custom-silicon/networking demand tailwind.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>ETN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D15" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E15" s="27" t="n">
         <v>412.97</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F15" s="35" t="inlineStr">
         <is>
           <t>Q2 2026 EPS/revenue beat, record 23.1% margin, backlog +43% YoY. Data-center power/cooling demand confirms XLI thesis.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>COF</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C16" s="36" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D16" s="23" t="n">
         <v>23</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E16" s="13" t="n">
         <v>216.96</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F16" s="33" t="inlineStr">
         <is>
           <t>Q2 2026 revenue +26% YoY; P/E compressed to ~12.2x. Discover acquisition integration driving growth. Diversification outside AI-infrastructure theme.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>AGG</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" s="34" t="inlineStr">
         <is>
           <t>BUY</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" s="26" t="n">
         <v>82</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E17" s="27" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F17" s="35" t="inlineStr">
         <is>
           <t>Passive core bond sleeve per fixed sizing rules, ~4.06% dividend yield.</t>
         </is>
@@ -2020,7 +2442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2029,135 +2451,158 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>CHARTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>% NAV</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>AI-Capex</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B4" s="16" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B5" s="15" t="n">
         <v>0.0499</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Healthcare-GLP1</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B6" s="16" t="n">
         <v>0.0486</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Consumer-Defensive</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B7" s="15" t="n">
         <v>0.09859999999999999</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Energy-Transition</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B8" s="16" t="n">
         <v>0.1593</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B9" s="15" t="n">
         <v>0.0497</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Diversified-Core</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B10" s="16" t="n">
         <v>0.0803</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Cycle Date</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>NAV</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Blended Benchmark</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B27" s="13" t="n">
         <v>100000</v>
       </c>
-      <c r="D12" t="n">
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="23" t="n">
         <v>766.08</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B28" s="27" t="n">
         <v>100000</v>
       </c>
-      <c r="D13" t="n">
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="26" t="n">
         <v>766.08</v>
       </c>
     </row>

</xml_diff>